<commit_message>
Deploying to gh-pages from @ NIH-NCPI/ncpi-fhir-ig-2@f67d595363e08834810088484fc3165e85fface9 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-consanguinity.xlsx
+++ b/StructureDefinition-consanguinity.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-12-03T22:26:51+00:00</t>
+    <t>2026-01-13T18:03:13+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Extension containing a consanguinity assertion</t>
+    <t>Extension containing Consanguinity</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -129,7 +129,7 @@
     <t>Context</t>
   </si>
   <si>
-    <t>element:Group</t>
+    <t>element:Element</t>
   </si>
   <si>
     <t>ID</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ NIH-NCPI/ncpi-fhir-ig-2@d51a350c79318d93b13f267eff80d597844c00bd 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-consanguinity.xlsx
+++ b/StructureDefinition-consanguinity.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-06T18:07:39+00:00</t>
+    <t>2026-03-09T20:11:59+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Extension containing Consanguinity</t>
+    <t>Extension containing a consanguinity assertion</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -129,7 +129,7 @@
     <t>Context</t>
   </si>
   <si>
-    <t>element:Element</t>
+    <t>element:Group</t>
   </si>
   <si>
     <t>ID</t>

</xml_diff>